<commit_message>
Round Bilanzgewinn to avoid floating point display artefact
Die Zeile "21. Bilanzgewinn" zeigte je nach Auswertungsreihenfolge (0.0)
statt des Nullstrichs, weil die Umrechnung von T€ in Mio. € einen
Gleitkommarest von rund 1e-15 hinterlaesst und das Zahlenformat den
Null-Zweig dann nicht trifft. Die Formel rundet jetzt auf sechs
Nachkommastellen; der ausgewiesene Wert bleibt unveraendert.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DtU8vczdxxth9TyTsDKbpL
</commit_message>
<xml_diff>
--- a/ESWE_Versorgungs_AG_Financial_Model_2021_2025.xlsx
+++ b/ESWE_Versorgungs_AG_Financial_Model_2021_2025.xlsx
@@ -4191,23 +4191,23 @@
         </is>
       </c>
       <c r="C29" s="40">
-        <f>C24-SUM(C26:C28)</f>
+        <f>ROUND(C24-SUM(C26:C28),6)</f>
         <v/>
       </c>
       <c r="D29" s="40">
-        <f>D24-SUM(D26:D28)</f>
+        <f>ROUND(D24-SUM(D26:D28),6)</f>
         <v/>
       </c>
       <c r="E29" s="40">
-        <f>E24-SUM(E26:E28)</f>
+        <f>ROUND(E24-SUM(E26:E28),6)</f>
         <v/>
       </c>
       <c r="F29" s="40">
-        <f>F24-SUM(F26:F28)</f>
+        <f>ROUND(F24-SUM(F26:F28),6)</f>
         <v/>
       </c>
       <c r="G29" s="40">
-        <f>G24-SUM(G26:G28)</f>
+        <f>ROUND(G24-SUM(G26:G28),6)</f>
         <v/>
       </c>
     </row>

</xml_diff>